<commit_message>
feat: tableros (boards + sections), task priority/subtasks/comments with @mentions, standup mode, task notifications
- Migration 20260910220000: boards/board_members/board_sections/board_tasks,
  tasks.workspace_id/priority/parent_task_id (objective_id nullable), comments.task_id/mentions,
  task_activity trail, trigger-based notifications (assigned/blocked/mention),
  notifications added to realtime publication, seeded Sprint/Backlog/Iniciativas boards
- Boards index + Kanban board page (dnd-kit), toolbar (Asignado, Filtros, Ordenar, Agrupar), Standup mode
- Task detail: Prioridad, Tableros block, Subtareas, Comentarios+Actividad, full-page /tareas/[id]
- Mis Tareas for members with quick filters; sidebar Tableros section
- CSP: allow unsafe-eval in development only (Next dev hydration)
- Docs: SCHEMA.md, CLAUDE.md, feature inventory xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Inventario-funcionalidades-Kublau-OKR.xlsx
+++ b/docs/Inventario-funcionalidades-Kublau-OKR.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Inventario" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Inventario!$A$1:$H$258</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Inventario!$A$1:$H$259</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2155" uniqueCount="1039">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2163" uniqueCount="1042">
   <si>
     <t xml:space="preserve">Estado</t>
   </si>
@@ -2418,6 +2418,303 @@
     <t xml:space="preserve">F-193</t>
   </si>
   <si>
+    <t xml:space="preserve">Sección "Tableros" bajo Funcionalidades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lista de tableros del workspace (favoritos primero) + "+ Nuevo tablero"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · Diseño ronda 1 A · cubre Asana: Projects, My tasks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entidades boards / board_sections / board_tasks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tablero (nombre, color, visibilidad workspace/privado, owner, depto), secciones con orden, colocación tarea-por-tablero con una sección por tablero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tasks + workspace_id, objective_id nullable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-195</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tablero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vista Kanban: secciones = columnas creadas por el usuario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contador por columna, menú ··· (renombrar, mover, ocultar vacías, eliminar → tareas a "Sin sección"), "+ Agregar sección" al final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · Cubre Asana: Sections, Board view</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-196</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drag &amp; drop de tarjetas entre secciones y reorden de secciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mover tarjeta = cambiar sección; el estado de la tarea no cambia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sección ≠ estado (decisión)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-197</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarjeta: título, chip prioridad, chip estado, objetivo, fecha (roja si vencida), avatar, contadores subtareas/comentarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumen de la tarea en la columna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-198</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Botón "+ Agregar tarea" (toolbar y pie de columna)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crea tarea en el tablero/sección; objetivo opcional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-199</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toolbar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dropdown "Asignado" separado del botón Filtros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtra el tablero por responsable con un clic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decisión del usuario: control independiente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Botón "Filtros: N" (chips rápidos + constructor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incompletas / Solo mías / Vencidas / Sin objetivo + por estado, prioridad, fecha, objetivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · Cubre Asana: Filters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Botón "Ordenar"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por prioridad, fecha límite, estado, responsable, alfabético (dentro de cada sección)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · Cubre Asana: Sort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Botón "Agrupar"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columnas por Sección (default), Estado o Responsable sin alterar las secciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · Cubre Asana: Group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Botón "Standup" (toggle)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entra/sale del modo Standup; también Esc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · Diseño ronda 2 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modo Standup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pantalla completa sin sidebar ni topbar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fullscreen API; barra mínima con nombre del tablero, fecha y "N de M han hablado" + botón Salir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo vista: no escribe nada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rail izquierdo con pila de personas del tablero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un botón por miembro con avatar, nombre y "N tareas · N vencidas"; agarre ⋮⋮ para reordenar (orden local al navegador)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clic en persona = filtrar Kanban a sus tareas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muestra solo las tareas asignadas a esa persona; secciones vacías se ocultan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado "ya habló" (check verde) al hacer clic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La persona clicada queda marcada; la actual resaltada; clic de nuevo desmarca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se descarta al salir del modo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-208</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kanban ampliado (+20% tipografía y tarjetas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legible en proyector/TV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clic en tarjeta abre el panel de detalle normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-209</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo "Prioridad" (Alta / Media / Baja)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chip de color editable inline y en el formulario; visible en tarjeta y fila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · MVP #1 · cubre Asana: Priority</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloque "Tableros"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lista de tableros donde vive la tarea con selector de sección inline + "Agregar a tablero"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como bloque Projects de Asana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-211</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sección "Subtareas" con contador N/M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checklist con asignado y fecha propios; barra de progreso; contador en tarjeta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · MVP #7 · parent_task_id · cubre Asana: Subtasks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sección "Comentarios" en tareas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hilo de comentarios en la tarea (reusa comments + task_id); toggle Comentarios / Actividad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · MVP #2 · cubre Asana: comentarios en tarea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-213</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@menciones en comentarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typeahead de miembros del workspace; mención resaltada; "Se notificará a N personas"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · MVP #2 · cubre Asana: @mention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-214</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Botón "⤢ Abrir" (página completa de la tarea)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abre la tarea en su propia URL con actividad tipo chat, seguidores y acciones Duplicar/Copiar enlace/Eliminar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · Diseño ronda 1 D · URL compartible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actividad automática en la tarea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eventos: cambio de prioridad, estado, sección, tablero, asignación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En cursiva dentro del hilo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-216</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emitir "tarea asignada", "tarea bloqueada", "mención en comentario"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aviso in-app en tiempo real (tipos ya existen) + email opcional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · MVP #3 · plumbing ya existe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-217</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mis Tareas visible para miembros (chips de filtro, orden por prioridad, panel de detalle)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hub personal cruzado de tableros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-10 · MVP #8 · cubre Asana: My tasks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-218</t>
+  </si>
+  <si>
     <t xml:space="preserve">CTA inline entre secciones</t>
   </si>
   <si>
@@ -2427,7 +2724,7 @@
     <t xml:space="preserve">Solicitud pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">F-194</t>
+    <t xml:space="preserve">F-219</t>
   </si>
   <si>
     <t xml:space="preserve">Guardado atómico del check-in</t>
@@ -2439,76 +2736,7 @@
     <t xml:space="preserve">Hallazgo P0 de auditoría</t>
   </si>
   <si>
-    <t xml:space="preserve">F-195</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sección "Tableros" bajo Funcionalidades</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lista de tableros del workspace (favoritos primero) + "+ Nuevo tablero"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diseño ronda 1 A · cubre Asana: Projects, My tasks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-196</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entidades boards / board_sections / board_tasks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tablero (nombre, color, visibilidad workspace/privado, owner, depto), secciones con orden, colocación tarea-por-tablero con una sección por tablero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tasks + workspace_id, objective_id nullable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-197</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tablero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vista Kanban: secciones = columnas creadas por el usuario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contador por columna, menú ··· (renombrar, mover, ocultar vacías, eliminar → tareas a "Sin sección"), "+ Agregar sección" al final</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubre Asana: Sections, Board view</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-198</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drag &amp; drop de tarjetas entre secciones y reorden de secciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mover tarjeta = cambiar sección; el estado de la tarea no cambia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sección ≠ estado (decisión)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-199</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarjeta: título, chip prioridad, chip estado, objetivo, fecha (roja si vencida), avatar, contadores subtareas/comentarios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resumen de la tarea en la columna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Botón "+ Agregar tarea" (toolbar y pie de columna)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crea tarea en el tablero/sección; objetivo opcional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-201</t>
+    <t xml:space="preserve">F-220</t>
   </si>
   <si>
     <t xml:space="preserve">Tabs Tablero / Lista / Calendario</t>
@@ -2520,58 +2748,7 @@
     <t xml:space="preserve">Lista y Calendario en fase posterior</t>
   </si>
   <si>
-    <t xml:space="preserve">F-202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toolbar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dropdown "Asignado" separado del botón Filtros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filtra el tablero por responsable con un clic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decisión del usuario: control independiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-203</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Botón "Filtros: N" (chips rápidos + constructor)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incompletas / Solo mías / Vencidas / Sin objetivo + por estado, prioridad, fecha, objetivo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubre Asana: Filters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Botón "Ordenar"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Por prioridad, fecha límite, estado, responsable, alfabético (dentro de cada sección)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubre Asana: Sort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-205</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Botón "Agrupar"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Columnas por Sección (default), Estado o Responsable sin alterar las secciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubre Asana: Group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-206</t>
+    <t xml:space="preserve">F-221</t>
   </si>
   <si>
     <t xml:space="preserve">Botón "Opciones"</t>
@@ -2583,136 +2760,7 @@
     <t xml:space="preserve">Fase posterior</t>
   </si>
   <si>
-    <t xml:space="preserve">F-207</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Botón "Standup" (toggle)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entra/sale del modo Standup; también Esc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diseño ronda 2 A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-208</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modo Standup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pantalla completa sin sidebar ni topbar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fullscreen API; barra mínima con nombre del tablero, fecha y "N de M han hablado" + botón Salir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solo vista: no escribe nada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-209</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rail izquierdo con pila de personas del tablero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un botón por miembro con avatar, nombre y "N tareas · N vencidas"; agarre ⋮⋮ para reordenar (orden local al navegador)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clic en persona = filtrar Kanban a sus tareas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muestra solo las tareas asignadas a esa persona; secciones vacías se ocultan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-211</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estado "ya habló" (check verde) al hacer clic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La persona clicada queda marcada; la actual resaltada; clic de nuevo desmarca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se descarta al salir del modo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-212</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kanban ampliado (+20% tipografía y tarjetas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legible en proyector/TV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clic en tarjeta abre el panel de detalle normal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-213</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo "Prioridad" (Alta / Media / Baja)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chip de color editable inline y en el formulario; visible en tarjeta y fila</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVP #1 · cubre Asana: Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-214</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bloque "Tableros"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lista de tableros donde vive la tarea con selector de sección inline + "Agregar a tablero"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como bloque Projects de Asana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-215</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sección "Subtareas" con contador N/M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checklist con asignado y fecha propios; barra de progreso; contador en tarjeta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVP #7 · parent_task_id · cubre Asana: Subtasks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-216</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sección "Comentarios" en tareas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hilo de comentarios en la tarea (reusa comments + task_id); toggle Comentarios / Actividad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVP #2 · cubre Asana: comentarios en tarea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-217</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@menciones en comentarios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typeahead de miembros del workspace; mención resaltada; "Se notificará a N personas"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVP #2 · cubre Asana: @mention</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-218</t>
+    <t xml:space="preserve">F-222</t>
   </si>
   <si>
     <t xml:space="preserve">Reacciones 👍 y "Responder"</t>
@@ -2721,57 +2769,18 @@
     <t xml:space="preserve">Reacción rápida y respuesta en hilo</t>
   </si>
   <si>
-    <t xml:space="preserve">F-219</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Botón "⤢ Abrir" (página completa de la tarea)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abre la tarea en su propia URL con actividad tipo chat, seguidores y acciones Duplicar/Copiar enlace/Eliminar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diseño ronda 1 D · URL compartible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-220</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Actividad automática en la tarea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eventos: cambio de prioridad, estado, sección, tablero, asignación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En cursiva dentro del hilo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-221</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emitir "tarea asignada", "tarea bloqueada", "mención en comentario"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aviso in-app en tiempo real (tipos ya existen) + email opcional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVP #3 · plumbing ya existe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-222</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mis Tareas visible para miembros + tabs Tablero/Calendario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hub personal cruzado de tableros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVP #8 · cubre Asana: My tasks</t>
-  </si>
-  <si>
     <t xml:space="preserve">F-223</t>
   </si>
   <si>
+    <t xml:space="preserve">Tabs Tablero / Calendario en Mis Tareas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vistas alternativas del hub personal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-224</t>
+  </si>
+  <si>
     <t xml:space="preserve">Detalle de tarea</t>
   </si>
   <si>
@@ -2781,7 +2790,7 @@
     <t xml:space="preserve">Toggle de completado; tipos Tarea, Hito, Aprobación (Aprobar / Solicitar cambios / Rechazar) con "Convertir a"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-224</t>
+    <t xml:space="preserve">F-225</t>
   </si>
   <si>
     <t xml:space="preserve">Campo Estado personalizado</t>
@@ -2790,7 +2799,7 @@
     <t xml:space="preserve">On track / At risk / Off track / On hold como chips de color, separado de "completada"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-225</t>
+    <t xml:space="preserve">F-226</t>
   </si>
   <si>
     <t xml:space="preserve">Asignado (único) con typeahead</t>
@@ -2802,7 +2811,7 @@
     <t xml:space="preserve">Auto-agrega a "My tasks" del asignado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-226</t>
+    <t xml:space="preserve">F-227</t>
   </si>
   <si>
     <t xml:space="preserve">Colaboradores / seguidores</t>
@@ -2814,7 +2823,7 @@
     <t xml:space="preserve">Vista previa "N people will be notified"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-227</t>
+    <t xml:space="preserve">F-228</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha límite con fecha inicio, hora y recurrencia</t>
@@ -2823,7 +2832,7 @@
     <t xml:space="preserve">Selector de rango; vencida en rojo en la tarjeta</t>
   </si>
   <si>
-    <t xml:space="preserve">F-228</t>
+    <t xml:space="preserve">F-229</t>
   </si>
   <si>
     <t xml:space="preserve">Dependencias "Blocked by" / "Blocking"</t>
@@ -2832,7 +2841,7 @@
     <t xml:space="preserve">Vincula tareas entre proyectos; se dibujan en Timeline</t>
   </si>
   <si>
-    <t xml:space="preserve">F-229</t>
+    <t xml:space="preserve">F-230</t>
   </si>
   <si>
     <t xml:space="preserve">Multi-proyecto (multi-homing)</t>
@@ -2841,7 +2850,7 @@
     <t xml:space="preserve">Una tarea vive en N proyectos, cada uno con su selector de sección inline</t>
   </si>
   <si>
-    <t xml:space="preserve">F-230</t>
+    <t xml:space="preserve">F-231</t>
   </si>
   <si>
     <t xml:space="preserve">Campos personalizados por proyecto</t>
@@ -2853,7 +2862,7 @@
     <t xml:space="preserve">"Edit options" y "Auto-fill" (IA) desde el dropdown</t>
   </si>
   <si>
-    <t xml:space="preserve">F-231</t>
+    <t xml:space="preserve">F-232</t>
   </si>
   <si>
     <t xml:space="preserve">Descripción rich text</t>
@@ -2862,7 +2871,7 @@
     <t xml:space="preserve">Editor con formato</t>
   </si>
   <si>
-    <t xml:space="preserve">F-232</t>
+    <t xml:space="preserve">F-233</t>
   </si>
   <si>
     <t xml:space="preserve">Subtareas</t>
@@ -2871,7 +2880,7 @@
     <t xml:space="preserve">Lista inline con contador "0/1", asignado y fecha propios, detalle anidado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-233</t>
+    <t xml:space="preserve">F-234</t>
   </si>
   <si>
     <t xml:space="preserve">Adjuntos</t>
@@ -2880,7 +2889,7 @@
     <t xml:space="preserve">Archivos adjuntos a la tarea</t>
   </si>
   <si>
-    <t xml:space="preserve">F-234</t>
+    <t xml:space="preserve">F-235</t>
   </si>
   <si>
     <t xml:space="preserve">Likes, copiar enlace, pantalla completa, banner de privacidad</t>
@@ -2892,7 +2901,7 @@
     <t xml:space="preserve">"Make public"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-235</t>
+    <t xml:space="preserve">F-236</t>
   </si>
   <si>
     <t xml:space="preserve">Menú "…" de tarea</t>
@@ -2907,7 +2916,7 @@
     <t xml:space="preserve">IA: Summarize task, Draft subtasks</t>
   </si>
   <si>
-    <t xml:space="preserve">F-236</t>
+    <t xml:space="preserve">F-237</t>
   </si>
   <si>
     <t xml:space="preserve">Feed de actividad</t>
@@ -2922,7 +2931,7 @@
     <t xml:space="preserve">Eventos: creado, renombrado (show original), asignado, campo cambiado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-237</t>
+    <t xml:space="preserve">F-238</t>
   </si>
   <si>
     <t xml:space="preserve">Editor</t>
@@ -2934,7 +2943,7 @@
     <t xml:space="preserve">Comentarios con formato completo</t>
   </si>
   <si>
-    <t xml:space="preserve">F-238</t>
+    <t xml:space="preserve">F-239</t>
   </si>
   <si>
     <t xml:space="preserve">@mención de personas, tareas y proyectos</t>
@@ -2943,7 +2952,7 @@
     <t xml:space="preserve">Typeahead en todo el workspace</t>
   </si>
   <si>
-    <t xml:space="preserve">F-239</t>
+    <t xml:space="preserve">F-240</t>
   </si>
   <si>
     <t xml:space="preserve">Comentario</t>
@@ -2955,7 +2964,7 @@
     <t xml:space="preserve">Acciones sobre cada comentario</t>
   </si>
   <si>
-    <t xml:space="preserve">F-240</t>
+    <t xml:space="preserve">F-241</t>
   </si>
   <si>
     <t xml:space="preserve">IA: resumir tarea, recomendar ediciones</t>
@@ -2964,7 +2973,7 @@
     <t xml:space="preserve">Asistencia en el compositor</t>
   </si>
   <si>
-    <t xml:space="preserve">F-241</t>
+    <t xml:space="preserve">F-242</t>
   </si>
   <si>
     <t xml:space="preserve">Board</t>
@@ -2976,7 +2985,7 @@
     <t xml:space="preserve">"Add section" inline al final; menú: rename, add before/after, collapse, hide empty, add rule, delete</t>
   </si>
   <si>
-    <t xml:space="preserve">F-242</t>
+    <t xml:space="preserve">F-243</t>
   </si>
   <si>
     <t xml:space="preserve">Drag &amp; drop entre secciones y reorden de secciones</t>
@@ -2985,7 +2994,7 @@
     <t xml:space="preserve">Mover tarea = cambiar sección</t>
   </si>
   <si>
-    <t xml:space="preserve">F-243</t>
+    <t xml:space="preserve">F-244</t>
   </si>
   <si>
     <t xml:space="preserve">Menú contextual de tarjeta (click derecho)</t>
@@ -2994,7 +3003,7 @@
     <t xml:space="preserve">Duplicar, follow-up, completar, subtarea, convertir, abrir en pestaña, copiar enlace, eliminar, imagen de portada</t>
   </si>
   <si>
-    <t xml:space="preserve">F-244</t>
+    <t xml:space="preserve">F-245</t>
   </si>
   <si>
     <t xml:space="preserve">Tarjeta con campos configurables</t>
@@ -3003,7 +3012,7 @@
     <t xml:space="preserve">Chips (Priority), fecha, tag, avatar, contadores like/comentario/subtarea</t>
   </si>
   <si>
-    <t xml:space="preserve">F-245</t>
+    <t xml:space="preserve">F-246</t>
   </si>
   <si>
     <t xml:space="preserve">Vistas</t>
@@ -3018,7 +3027,7 @@
     <t xml:space="preserve">List: una columna por campo, "+" agrega campo</t>
   </si>
   <si>
-    <t xml:space="preserve">F-246</t>
+    <t xml:space="preserve">F-247</t>
   </si>
   <si>
     <t xml:space="preserve">Filtros rápidos + constructor apilable</t>
@@ -3027,7 +3036,7 @@
     <t xml:space="preserve">Incomplete, Completed, Just my tasks, Due this/next week; por asignado, fechas, tipo y cada campo personalizado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-247</t>
+    <t xml:space="preserve">F-248</t>
   </si>
   <si>
     <t xml:space="preserve">Ordenar por cualquier campo</t>
@@ -3036,7 +3045,7 @@
     <t xml:space="preserve">Fechas, asignado, likes, alfabético, cada campo personalizado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-248</t>
+    <t xml:space="preserve">F-249</t>
   </si>
   <si>
     <t xml:space="preserve">Agrupar por cualquier campo + subgrupo (swimlanes)</t>
@@ -3045,7 +3054,7 @@
     <t xml:space="preserve">Agrupación distinta de secciones con orden personalizado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-249</t>
+    <t xml:space="preserve">F-250</t>
   </si>
   <si>
     <t xml:space="preserve">Panel "Options" por vista</t>
@@ -3054,7 +3063,7 @@
     <t xml:space="preserve">Mostrar/ocultar campos, subtareas colapsadas/expandidas, nombre/icono de vista</t>
   </si>
   <si>
-    <t xml:space="preserve">F-250</t>
+    <t xml:space="preserve">F-251</t>
   </si>
   <si>
     <t xml:space="preserve">Buscar en esta vista</t>
@@ -3063,7 +3072,7 @@
     <t xml:space="preserve">Búsqueda rápida</t>
   </si>
   <si>
-    <t xml:space="preserve">F-251</t>
+    <t xml:space="preserve">F-252</t>
   </si>
   <si>
     <t xml:space="preserve">Customize &gt; Fields</t>
@@ -3075,7 +3084,7 @@
     <t xml:space="preserve">Single-select, Multi-select, Date, People, Reference, Text, Number, Formula, ID, Timer, Time tracking, Rollup</t>
   </si>
   <si>
-    <t xml:space="preserve">F-252</t>
+    <t xml:space="preserve">F-253</t>
   </si>
   <si>
     <t xml:space="preserve">Biblioteca de campos del workspace</t>
@@ -3084,7 +3093,7 @@
     <t xml:space="preserve">Reusar campos entre proyectos; opciones con color; reordenar; IA "Recommend fields"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-253</t>
+    <t xml:space="preserve">F-254</t>
   </si>
   <si>
     <t xml:space="preserve">Customize &gt; Rules</t>
@@ -3099,7 +3108,7 @@
     <t xml:space="preserve">Plantillas de reglas con IA</t>
   </si>
   <si>
-    <t xml:space="preserve">F-254</t>
+    <t xml:space="preserve">F-255</t>
   </si>
   <si>
     <t xml:space="preserve">Customize</t>
@@ -3111,7 +3120,7 @@
     <t xml:space="preserve">Intake y plantillas</t>
   </si>
   <si>
-    <t xml:space="preserve">F-255</t>
+    <t xml:space="preserve">F-256</t>
   </si>
   <si>
     <t xml:space="preserve">Menú de proyecto</t>
@@ -3123,7 +3132,7 @@
     <t xml:space="preserve">Gestión del proyecto</t>
   </si>
   <si>
-    <t xml:space="preserve">F-256</t>
+    <t xml:space="preserve">F-257</t>
   </si>
   <si>
     <t xml:space="preserve">My tasks / Inbox</t>
@@ -3135,7 +3144,7 @@
     <t xml:space="preserve">Lista personal con secciones automáticas ("Recently assigned")</t>
   </si>
   <si>
-    <t xml:space="preserve">F-257</t>
+    <t xml:space="preserve">F-258</t>
   </si>
   <si>
     <t xml:space="preserve">Widgets de conteo y gráficas</t>
@@ -3956,11 +3965,11 @@
       </c>
       <c r="C10" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A10,Inventario!$F:$F,"Actual")</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D10" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A10,Inventario!$F:$F,"Futuro")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E10" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A10,Inventario!$F:$F,"Asana ahora")</f>
@@ -3968,7 +3977,7 @@
       </c>
       <c r="F10" s="8" t="n">
         <f aca="false">SUM(C10:E10)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4220,11 +4229,11 @@
       </c>
       <c r="C21" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A21,Inventario!$F:$F,"Actual")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D21" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A21,Inventario!$F:$F,"Futuro")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A21,Inventario!$F:$F,"Asana ahora")</f>
@@ -4364,11 +4373,11 @@
       </c>
       <c r="C27" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A27,Inventario!$F:$F,"Actual")</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="D27" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A27,Inventario!$F:$F,"Futuro")</f>
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E27" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A27,Inventario!$F:$F,"Asana ahora")</f>
@@ -4601,11 +4610,11 @@
       </c>
       <c r="C37" s="9" t="n">
         <f aca="false">SUM(C2:C36)</f>
-        <v>192</v>
+        <v>217</v>
       </c>
       <c r="D37" s="9" t="n">
         <f aca="false">SUM(D2:D36)</f>
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E37" s="9" t="n">
         <f aca="false">SUM(E2:E36)</f>
@@ -4613,7 +4622,7 @@
       </c>
       <c r="F37" s="9" t="n">
         <f aca="false">SUM(F2:F36)</f>
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -4632,7 +4641,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H258"/>
+  <dimension ref="A1:H259"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -9663,15 +9672,15 @@
         <v>98</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="8" t="s">
         <v>796</v>
       </c>
       <c r="B194" s="8" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C194" s="8" t="s">
-        <v>136</v>
+        <v>708</v>
       </c>
       <c r="D194" s="8" t="s">
         <v>797</v>
@@ -9679,25 +9688,25 @@
       <c r="E194" s="8" t="s">
         <v>798</v>
       </c>
-      <c r="F194" s="11" t="s">
-        <v>4</v>
+      <c r="F194" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G194" s="8" t="s">
-        <v>98</v>
+        <v>711</v>
       </c>
       <c r="H194" s="8" t="s">
         <v>799</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="8" t="s">
         <v>800</v>
       </c>
       <c r="B195" s="8" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C195" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D195" s="8" t="s">
         <v>801</v>
@@ -9705,8 +9714,8 @@
       <c r="E195" s="8" t="s">
         <v>802</v>
       </c>
-      <c r="F195" s="11" t="s">
-        <v>4</v>
+      <c r="F195" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G195" s="8" t="s">
         <v>98</v>
@@ -9723,59 +9732,59 @@
         <v>68</v>
       </c>
       <c r="C196" s="8" t="s">
-        <v>708</v>
+        <v>805</v>
       </c>
       <c r="D196" s="8" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="E196" s="8" t="s">
-        <v>806</v>
-      </c>
-      <c r="F196" s="11" t="s">
-        <v>4</v>
+        <v>807</v>
+      </c>
+      <c r="F196" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G196" s="8" t="s">
-        <v>711</v>
+        <v>291</v>
       </c>
       <c r="H196" s="8" t="s">
-        <v>807</v>
-      </c>
-    </row>
-    <row r="197" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="8" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="B197" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C197" s="8" t="s">
-        <v>66</v>
+        <v>805</v>
       </c>
       <c r="D197" s="8" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="E197" s="8" t="s">
-        <v>810</v>
-      </c>
-      <c r="F197" s="11" t="s">
-        <v>4</v>
+        <v>811</v>
+      </c>
+      <c r="F197" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G197" s="8" t="s">
-        <v>98</v>
+        <v>291</v>
       </c>
       <c r="H197" s="8" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="198" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="8" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="B198" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C198" s="8" t="s">
-        <v>813</v>
+        <v>805</v>
       </c>
       <c r="D198" s="8" t="s">
         <v>814</v>
@@ -9783,66 +9792,66 @@
       <c r="E198" s="8" t="s">
         <v>815</v>
       </c>
-      <c r="F198" s="11" t="s">
-        <v>4</v>
+      <c r="F198" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G198" s="8" t="s">
-        <v>291</v>
+        <v>98</v>
       </c>
       <c r="H198" s="8" t="s">
-        <v>816</v>
+        <v>98</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="8" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B199" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C199" s="8" t="s">
-        <v>813</v>
+        <v>805</v>
       </c>
       <c r="D199" s="8" t="s">
+        <v>817</v>
+      </c>
+      <c r="E199" s="8" t="s">
         <v>818</v>
       </c>
-      <c r="E199" s="8" t="s">
-        <v>819</v>
-      </c>
-      <c r="F199" s="11" t="s">
-        <v>4</v>
+      <c r="F199" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G199" s="8" t="s">
         <v>291</v>
       </c>
       <c r="H199" s="8" t="s">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="200" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="8" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="B200" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C200" s="8" t="s">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="D200" s="8" t="s">
+        <v>821</v>
+      </c>
+      <c r="E200" s="8" t="s">
         <v>822</v>
       </c>
-      <c r="E200" s="8" t="s">
+      <c r="F200" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G200" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H200" s="8" t="s">
         <v>823</v>
-      </c>
-      <c r="F200" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="G200" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="H200" s="8" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9853,7 +9862,7 @@
         <v>68</v>
       </c>
       <c r="C201" s="8" t="s">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="D201" s="8" t="s">
         <v>825</v>
@@ -9861,51 +9870,51 @@
       <c r="E201" s="8" t="s">
         <v>826</v>
       </c>
-      <c r="F201" s="11" t="s">
-        <v>4</v>
+      <c r="F201" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G201" s="8" t="s">
-        <v>291</v>
+        <v>98</v>
       </c>
       <c r="H201" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="8" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="B202" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C202" s="8" t="s">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="D202" s="8" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="E202" s="8" t="s">
-        <v>829</v>
-      </c>
-      <c r="F202" s="11" t="s">
-        <v>4</v>
+        <v>830</v>
+      </c>
+      <c r="F202" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G202" s="8" t="s">
         <v>98</v>
       </c>
       <c r="H202" s="8" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="8" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="B203" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C203" s="8" t="s">
-        <v>832</v>
+        <v>820</v>
       </c>
       <c r="D203" s="8" t="s">
         <v>833</v>
@@ -9913,8 +9922,8 @@
       <c r="E203" s="8" t="s">
         <v>834</v>
       </c>
-      <c r="F203" s="11" t="s">
-        <v>4</v>
+      <c r="F203" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G203" s="8" t="s">
         <v>98</v>
@@ -9931,7 +9940,7 @@
         <v>68</v>
       </c>
       <c r="C204" s="8" t="s">
-        <v>832</v>
+        <v>820</v>
       </c>
       <c r="D204" s="8" t="s">
         <v>837</v>
@@ -9939,11 +9948,11 @@
       <c r="E204" s="8" t="s">
         <v>838</v>
       </c>
-      <c r="F204" s="11" t="s">
-        <v>4</v>
+      <c r="F204" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G204" s="8" t="s">
-        <v>98</v>
+        <v>711</v>
       </c>
       <c r="H204" s="8" t="s">
         <v>839</v>
@@ -9957,51 +9966,51 @@
         <v>68</v>
       </c>
       <c r="C205" s="8" t="s">
-        <v>832</v>
+        <v>841</v>
       </c>
       <c r="D205" s="8" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="E205" s="8" t="s">
-        <v>842</v>
-      </c>
-      <c r="F205" s="11" t="s">
-        <v>4</v>
+        <v>843</v>
+      </c>
+      <c r="F205" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G205" s="8" t="s">
-        <v>98</v>
+        <v>711</v>
       </c>
       <c r="H205" s="8" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="8" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B206" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C206" s="8" t="s">
-        <v>832</v>
+        <v>841</v>
       </c>
       <c r="D206" s="8" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="E206" s="8" t="s">
-        <v>846</v>
-      </c>
-      <c r="F206" s="11" t="s">
-        <v>4</v>
+        <v>847</v>
+      </c>
+      <c r="F206" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G206" s="8" t="s">
-        <v>98</v>
+        <v>711</v>
       </c>
       <c r="H206" s="8" t="s">
-        <v>847</v>
-      </c>
-    </row>
-    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="8" t="s">
         <v>848</v>
       </c>
@@ -10009,7 +10018,7 @@
         <v>68</v>
       </c>
       <c r="C207" s="8" t="s">
-        <v>832</v>
+        <v>841</v>
       </c>
       <c r="D207" s="8" t="s">
         <v>849</v>
@@ -10017,118 +10026,118 @@
       <c r="E207" s="8" t="s">
         <v>850</v>
       </c>
-      <c r="F207" s="11" t="s">
-        <v>4</v>
+      <c r="F207" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G207" s="8" t="s">
-        <v>98</v>
+        <v>711</v>
       </c>
       <c r="H207" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="8" t="s">
         <v>851</v>
-      </c>
-    </row>
-    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A208" s="8" t="s">
-        <v>852</v>
       </c>
       <c r="B208" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C208" s="8" t="s">
-        <v>832</v>
+        <v>841</v>
       </c>
       <c r="D208" s="8" t="s">
+        <v>852</v>
+      </c>
+      <c r="E208" s="8" t="s">
         <v>853</v>
       </c>
-      <c r="E208" s="8" t="s">
-        <v>854</v>
-      </c>
-      <c r="F208" s="11" t="s">
-        <v>4</v>
+      <c r="F208" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G208" s="8" t="s">
         <v>711</v>
       </c>
       <c r="H208" s="8" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="8" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B209" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C209" s="8" t="s">
+        <v>841</v>
+      </c>
+      <c r="D209" s="8" t="s">
+        <v>856</v>
+      </c>
+      <c r="E209" s="8" t="s">
         <v>857</v>
       </c>
-      <c r="D209" s="8" t="s">
-        <v>858</v>
-      </c>
-      <c r="E209" s="8" t="s">
-        <v>859</v>
-      </c>
-      <c r="F209" s="11" t="s">
-        <v>4</v>
+      <c r="F209" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G209" s="8" t="s">
         <v>711</v>
       </c>
       <c r="H209" s="8" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="8" t="s">
+        <v>859</v>
+      </c>
+      <c r="B210" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C210" s="8" t="s">
+        <v>558</v>
+      </c>
+      <c r="D210" s="8" t="s">
+        <v>860</v>
+      </c>
+      <c r="E210" s="8" t="s">
         <v>861</v>
       </c>
-      <c r="B210" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C210" s="8" t="s">
-        <v>857</v>
-      </c>
-      <c r="D210" s="8" t="s">
+      <c r="F210" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G210" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="H210" s="8" t="s">
         <v>862</v>
-      </c>
-      <c r="E210" s="8" t="s">
-        <v>863</v>
-      </c>
-      <c r="F210" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="G210" s="8" t="s">
-        <v>711</v>
-      </c>
-      <c r="H210" s="8" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="8" t="s">
+        <v>863</v>
+      </c>
+      <c r="B211" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C211" s="8" t="s">
+        <v>558</v>
+      </c>
+      <c r="D211" s="8" t="s">
         <v>864</v>
       </c>
-      <c r="B211" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C211" s="8" t="s">
-        <v>857</v>
-      </c>
-      <c r="D211" s="8" t="s">
+      <c r="E211" s="8" t="s">
         <v>865</v>
       </c>
-      <c r="E211" s="8" t="s">
+      <c r="F211" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G211" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="H211" s="8" t="s">
         <v>866</v>
-      </c>
-      <c r="F211" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="G211" s="8" t="s">
-        <v>711</v>
-      </c>
-      <c r="H211" s="8" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10136,10 +10145,10 @@
         <v>867</v>
       </c>
       <c r="B212" s="8" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="C212" s="8" t="s">
-        <v>857</v>
+        <v>558</v>
       </c>
       <c r="D212" s="8" t="s">
         <v>868</v>
@@ -10147,11 +10156,11 @@
       <c r="E212" s="8" t="s">
         <v>869</v>
       </c>
-      <c r="F212" s="11" t="s">
-        <v>4</v>
+      <c r="F212" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G212" s="8" t="s">
-        <v>711</v>
+        <v>291</v>
       </c>
       <c r="H212" s="8" t="s">
         <v>870</v>
@@ -10162,10 +10171,10 @@
         <v>871</v>
       </c>
       <c r="B213" s="8" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="C213" s="8" t="s">
-        <v>857</v>
+        <v>558</v>
       </c>
       <c r="D213" s="8" t="s">
         <v>872</v>
@@ -10173,17 +10182,17 @@
       <c r="E213" s="8" t="s">
         <v>873</v>
       </c>
-      <c r="F213" s="11" t="s">
-        <v>4</v>
+      <c r="F213" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G213" s="8" t="s">
-        <v>711</v>
+        <v>98</v>
       </c>
       <c r="H213" s="8" t="s">
         <v>874</v>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="8" t="s">
         <v>875</v>
       </c>
@@ -10199,11 +10208,11 @@
       <c r="E214" s="8" t="s">
         <v>877</v>
       </c>
-      <c r="F214" s="11" t="s">
-        <v>4</v>
+      <c r="F214" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G214" s="8" t="s">
-        <v>291</v>
+        <v>98</v>
       </c>
       <c r="H214" s="8" t="s">
         <v>878</v>
@@ -10225,17 +10234,17 @@
       <c r="E215" s="8" t="s">
         <v>881</v>
       </c>
-      <c r="F215" s="11" t="s">
-        <v>4</v>
+      <c r="F215" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G215" s="8" t="s">
-        <v>291</v>
+        <v>98</v>
       </c>
       <c r="H215" s="8" t="s">
         <v>882</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="8" t="s">
         <v>883</v>
       </c>
@@ -10251,11 +10260,11 @@
       <c r="E216" s="8" t="s">
         <v>885</v>
       </c>
-      <c r="F216" s="11" t="s">
-        <v>4</v>
+      <c r="F216" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G216" s="8" t="s">
-        <v>291</v>
+        <v>98</v>
       </c>
       <c r="H216" s="8" t="s">
         <v>886</v>
@@ -10266,10 +10275,10 @@
         <v>887</v>
       </c>
       <c r="B217" s="8" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="C217" s="8" t="s">
-        <v>558</v>
+        <v>64</v>
       </c>
       <c r="D217" s="8" t="s">
         <v>888</v>
@@ -10277,11 +10286,11 @@
       <c r="E217" s="8" t="s">
         <v>889</v>
       </c>
-      <c r="F217" s="11" t="s">
-        <v>4</v>
+      <c r="F217" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G217" s="8" t="s">
-        <v>98</v>
+        <v>711</v>
       </c>
       <c r="H217" s="8" t="s">
         <v>890</v>
@@ -10295,7 +10304,7 @@
         <v>34</v>
       </c>
       <c r="C218" s="8" t="s">
-        <v>558</v>
+        <v>505</v>
       </c>
       <c r="D218" s="8" t="s">
         <v>892</v>
@@ -10303,11 +10312,11 @@
       <c r="E218" s="8" t="s">
         <v>893</v>
       </c>
-      <c r="F218" s="11" t="s">
-        <v>4</v>
+      <c r="F218" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G218" s="8" t="s">
-        <v>98</v>
+        <v>711</v>
       </c>
       <c r="H218" s="8" t="s">
         <v>894</v>
@@ -10318,10 +10327,10 @@
         <v>895</v>
       </c>
       <c r="B219" s="8" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C219" s="8" t="s">
-        <v>558</v>
+        <v>136</v>
       </c>
       <c r="D219" s="8" t="s">
         <v>896</v>
@@ -10336,24 +10345,24 @@
         <v>98</v>
       </c>
       <c r="H219" s="8" t="s">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="220" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="8" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="B220" s="8" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C220" s="8" t="s">
-        <v>558</v>
+        <v>64</v>
       </c>
       <c r="D220" s="8" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="E220" s="8" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="F220" s="11" t="s">
         <v>4</v>
@@ -10362,24 +10371,24 @@
         <v>98</v>
       </c>
       <c r="H220" s="8" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="8" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="B221" s="8" t="s">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="C221" s="8" t="s">
-        <v>558</v>
+        <v>805</v>
       </c>
       <c r="D221" s="8" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="E221" s="8" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="F221" s="11" t="s">
         <v>4</v>
@@ -10388,96 +10397,96 @@
         <v>98</v>
       </c>
       <c r="H221" s="8" t="s">
-        <v>905</v>
-      </c>
-    </row>
-    <row r="222" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="8" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="B222" s="8" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="C222" s="8" t="s">
-        <v>64</v>
+        <v>820</v>
       </c>
       <c r="D222" s="8" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="E222" s="8" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="F222" s="11" t="s">
         <v>4</v>
       </c>
       <c r="G222" s="8" t="s">
-        <v>711</v>
+        <v>98</v>
       </c>
       <c r="H222" s="8" t="s">
-        <v>909</v>
-      </c>
-    </row>
-    <row r="223" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="8" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="B223" s="8" t="s">
         <v>34</v>
       </c>
       <c r="C223" s="8" t="s">
-        <v>505</v>
+        <v>558</v>
       </c>
       <c r="D223" s="8" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="E223" s="8" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="F223" s="11" t="s">
         <v>4</v>
       </c>
       <c r="G223" s="8" t="s">
-        <v>711</v>
+        <v>98</v>
       </c>
       <c r="H223" s="8" t="s">
-        <v>913</v>
-      </c>
-    </row>
-    <row r="224" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="8" t="s">
         <v>914</v>
       </c>
       <c r="B224" s="8" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="C224" s="8" t="s">
+        <v>505</v>
+      </c>
+      <c r="D224" s="8" t="s">
         <v>915</v>
       </c>
-      <c r="D224" s="8" t="s">
+      <c r="E224" s="8" t="s">
         <v>916</v>
       </c>
-      <c r="E224" s="8" t="s">
-        <v>917</v>
-      </c>
-      <c r="F224" s="12" t="s">
-        <v>6</v>
+      <c r="F224" s="11" t="s">
+        <v>4</v>
       </c>
       <c r="G224" s="8" t="s">
-        <v>98</v>
+        <v>4</v>
       </c>
       <c r="H224" s="8" t="s">
-        <v>98</v>
+        <v>711</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="8" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="B225" s="8" t="s">
         <v>70</v>
       </c>
       <c r="C225" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D225" s="8" t="s">
         <v>919</v>
@@ -10503,7 +10512,7 @@
         <v>70</v>
       </c>
       <c r="C226" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D226" s="8" t="s">
         <v>922</v>
@@ -10518,24 +10527,24 @@
         <v>98</v>
       </c>
       <c r="H226" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="8" t="s">
         <v>924</v>
-      </c>
-    </row>
-    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A227" s="8" t="s">
-        <v>925</v>
       </c>
       <c r="B227" s="8" t="s">
         <v>70</v>
       </c>
       <c r="C227" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D227" s="8" t="s">
+        <v>925</v>
+      </c>
+      <c r="E227" s="8" t="s">
         <v>926</v>
-      </c>
-      <c r="E227" s="8" t="s">
-        <v>927</v>
       </c>
       <c r="F227" s="12" t="s">
         <v>6</v>
@@ -10544,24 +10553,24 @@
         <v>98</v>
       </c>
       <c r="H227" s="8" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="8" t="s">
         <v>928</v>
-      </c>
-    </row>
-    <row r="228" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A228" s="8" t="s">
-        <v>929</v>
       </c>
       <c r="B228" s="8" t="s">
         <v>70</v>
       </c>
       <c r="C228" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D228" s="8" t="s">
+        <v>929</v>
+      </c>
+      <c r="E228" s="8" t="s">
         <v>930</v>
-      </c>
-      <c r="E228" s="8" t="s">
-        <v>931</v>
       </c>
       <c r="F228" s="12" t="s">
         <v>6</v>
@@ -10570,10 +10579,10 @@
         <v>98</v>
       </c>
       <c r="H228" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="8" t="s">
         <v>932</v>
       </c>
@@ -10581,7 +10590,7 @@
         <v>70</v>
       </c>
       <c r="C229" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D229" s="8" t="s">
         <v>933</v>
@@ -10607,7 +10616,7 @@
         <v>70</v>
       </c>
       <c r="C230" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D230" s="8" t="s">
         <v>936</v>
@@ -10625,7 +10634,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="8" t="s">
         <v>938</v>
       </c>
@@ -10633,7 +10642,7 @@
         <v>70</v>
       </c>
       <c r="C231" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D231" s="8" t="s">
         <v>939</v>
@@ -10648,24 +10657,24 @@
         <v>98</v>
       </c>
       <c r="H231" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="8" t="s">
         <v>941</v>
-      </c>
-    </row>
-    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A232" s="8" t="s">
-        <v>942</v>
       </c>
       <c r="B232" s="8" t="s">
         <v>70</v>
       </c>
       <c r="C232" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D232" s="8" t="s">
+        <v>942</v>
+      </c>
+      <c r="E232" s="8" t="s">
         <v>943</v>
-      </c>
-      <c r="E232" s="8" t="s">
-        <v>944</v>
       </c>
       <c r="F232" s="12" t="s">
         <v>6</v>
@@ -10674,7 +10683,7 @@
         <v>98</v>
       </c>
       <c r="H232" s="8" t="s">
-        <v>98</v>
+        <v>944</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10685,7 +10694,7 @@
         <v>70</v>
       </c>
       <c r="C233" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D233" s="8" t="s">
         <v>946</v>
@@ -10711,7 +10720,7 @@
         <v>70</v>
       </c>
       <c r="C234" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D234" s="8" t="s">
         <v>949</v>
@@ -10729,7 +10738,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="8" t="s">
         <v>951</v>
       </c>
@@ -10737,7 +10746,7 @@
         <v>70</v>
       </c>
       <c r="C235" s="8" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="D235" s="8" t="s">
         <v>952</v>
@@ -10752,24 +10761,24 @@
         <v>98</v>
       </c>
       <c r="H235" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="8" t="s">
         <v>954</v>
-      </c>
-    </row>
-    <row r="236" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A236" s="8" t="s">
-        <v>955</v>
       </c>
       <c r="B236" s="8" t="s">
         <v>70</v>
       </c>
       <c r="C236" s="8" t="s">
+        <v>918</v>
+      </c>
+      <c r="D236" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="E236" s="8" t="s">
         <v>956</v>
-      </c>
-      <c r="D236" s="8" t="s">
-        <v>957</v>
-      </c>
-      <c r="E236" s="8" t="s">
-        <v>958</v>
       </c>
       <c r="F236" s="12" t="s">
         <v>6</v>
@@ -10778,24 +10787,24 @@
         <v>98</v>
       </c>
       <c r="H236" s="8" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="8" t="s">
+        <v>958</v>
+      </c>
+      <c r="B237" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C237" s="8" t="s">
         <v>959</v>
       </c>
-    </row>
-    <row r="237" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A237" s="8" t="s">
+      <c r="D237" s="8" t="s">
         <v>960</v>
       </c>
-      <c r="B237" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C237" s="8" t="s">
+      <c r="E237" s="8" t="s">
         <v>961</v>
-      </c>
-      <c r="D237" s="8" t="s">
-        <v>962</v>
-      </c>
-      <c r="E237" s="8" t="s">
-        <v>963</v>
       </c>
       <c r="F237" s="12" t="s">
         <v>6</v>
@@ -10804,24 +10813,24 @@
         <v>98</v>
       </c>
       <c r="H237" s="8" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="8" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="B238" s="8" t="s">
         <v>72</v>
       </c>
       <c r="C238" s="8" t="s">
+        <v>964</v>
+      </c>
+      <c r="D238" s="8" t="s">
+        <v>965</v>
+      </c>
+      <c r="E238" s="8" t="s">
         <v>966</v>
-      </c>
-      <c r="D238" s="8" t="s">
-        <v>967</v>
-      </c>
-      <c r="E238" s="8" t="s">
-        <v>968</v>
       </c>
       <c r="F238" s="12" t="s">
         <v>6</v>
@@ -10830,18 +10839,18 @@
         <v>98</v>
       </c>
       <c r="H238" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="239" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="8" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B239" s="8" t="s">
         <v>72</v>
       </c>
       <c r="C239" s="8" t="s">
-        <v>966</v>
+        <v>969</v>
       </c>
       <c r="D239" s="8" t="s">
         <v>970</v>
@@ -10859,7 +10868,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="240" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="8" t="s">
         <v>972</v>
       </c>
@@ -10867,13 +10876,13 @@
         <v>72</v>
       </c>
       <c r="C240" s="8" t="s">
+        <v>969</v>
+      </c>
+      <c r="D240" s="8" t="s">
         <v>973</v>
       </c>
-      <c r="D240" s="8" t="s">
+      <c r="E240" s="8" t="s">
         <v>974</v>
-      </c>
-      <c r="E240" s="8" t="s">
-        <v>975</v>
       </c>
       <c r="F240" s="12" t="s">
         <v>6</v>
@@ -10885,15 +10894,15 @@
         <v>98</v>
       </c>
     </row>
-    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="241" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="8" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B241" s="8" t="s">
         <v>72</v>
       </c>
       <c r="C241" s="8" t="s">
-        <v>966</v>
+        <v>976</v>
       </c>
       <c r="D241" s="8" t="s">
         <v>977</v>
@@ -10911,21 +10920,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="8" t="s">
         <v>979</v>
       </c>
       <c r="B242" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C242" s="8" t="s">
+        <v>969</v>
+      </c>
+      <c r="D242" s="8" t="s">
         <v>980</v>
       </c>
-      <c r="D242" s="8" t="s">
+      <c r="E242" s="8" t="s">
         <v>981</v>
-      </c>
-      <c r="E242" s="8" t="s">
-        <v>982</v>
       </c>
       <c r="F242" s="12" t="s">
         <v>6</v>
@@ -10939,13 +10948,13 @@
     </row>
     <row r="243" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="8" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B243" s="8" t="s">
         <v>74</v>
       </c>
       <c r="C243" s="8" t="s">
-        <v>980</v>
+        <v>983</v>
       </c>
       <c r="D243" s="8" t="s">
         <v>984</v>
@@ -10971,7 +10980,7 @@
         <v>74</v>
       </c>
       <c r="C244" s="8" t="s">
-        <v>980</v>
+        <v>983</v>
       </c>
       <c r="D244" s="8" t="s">
         <v>987</v>
@@ -10989,7 +10998,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="245" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="8" t="s">
         <v>989</v>
       </c>
@@ -10997,7 +11006,7 @@
         <v>74</v>
       </c>
       <c r="C245" s="8" t="s">
-        <v>980</v>
+        <v>983</v>
       </c>
       <c r="D245" s="8" t="s">
         <v>990</v>
@@ -11015,7 +11024,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="246" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="8" t="s">
         <v>992</v>
       </c>
@@ -11023,13 +11032,13 @@
         <v>74</v>
       </c>
       <c r="C246" s="8" t="s">
+        <v>983</v>
+      </c>
+      <c r="D246" s="8" t="s">
         <v>993</v>
       </c>
-      <c r="D246" s="8" t="s">
+      <c r="E246" s="8" t="s">
         <v>994</v>
-      </c>
-      <c r="E246" s="8" t="s">
-        <v>995</v>
       </c>
       <c r="F246" s="12" t="s">
         <v>6</v>
@@ -11038,24 +11047,24 @@
         <v>98</v>
       </c>
       <c r="H246" s="8" t="s">
-        <v>996</v>
+        <v>98</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="8" t="s">
+        <v>995</v>
+      </c>
+      <c r="B247" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C247" s="8" t="s">
+        <v>996</v>
+      </c>
+      <c r="D247" s="8" t="s">
         <v>997</v>
       </c>
-      <c r="B247" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C247" s="8" t="s">
-        <v>832</v>
-      </c>
-      <c r="D247" s="8" t="s">
+      <c r="E247" s="8" t="s">
         <v>998</v>
-      </c>
-      <c r="E247" s="8" t="s">
-        <v>999</v>
       </c>
       <c r="F247" s="12" t="s">
         <v>6</v>
@@ -11064,10 +11073,10 @@
         <v>98</v>
       </c>
       <c r="H247" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="248" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="8" t="s">
         <v>1000</v>
       </c>
@@ -11075,7 +11084,7 @@
         <v>76</v>
       </c>
       <c r="C248" s="8" t="s">
-        <v>832</v>
+        <v>820</v>
       </c>
       <c r="D248" s="8" t="s">
         <v>1001</v>
@@ -11093,7 +11102,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="249" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="8" t="s">
         <v>1003</v>
       </c>
@@ -11101,7 +11110,7 @@
         <v>76</v>
       </c>
       <c r="C249" s="8" t="s">
-        <v>832</v>
+        <v>820</v>
       </c>
       <c r="D249" s="8" t="s">
         <v>1004</v>
@@ -11127,7 +11136,7 @@
         <v>76</v>
       </c>
       <c r="C250" s="8" t="s">
-        <v>832</v>
+        <v>820</v>
       </c>
       <c r="D250" s="8" t="s">
         <v>1007</v>
@@ -11145,7 +11154,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="251" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="8" t="s">
         <v>1009</v>
       </c>
@@ -11153,7 +11162,7 @@
         <v>76</v>
       </c>
       <c r="C251" s="8" t="s">
-        <v>832</v>
+        <v>820</v>
       </c>
       <c r="D251" s="8" t="s">
         <v>1010</v>
@@ -11171,21 +11180,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="252" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="8" t="s">
         <v>1012</v>
       </c>
       <c r="B252" s="8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C252" s="8" t="s">
+        <v>820</v>
+      </c>
+      <c r="D252" s="8" t="s">
         <v>1013</v>
       </c>
-      <c r="D252" s="8" t="s">
+      <c r="E252" s="8" t="s">
         <v>1014</v>
-      </c>
-      <c r="E252" s="8" t="s">
-        <v>1015</v>
       </c>
       <c r="F252" s="12" t="s">
         <v>6</v>
@@ -11199,13 +11208,13 @@
     </row>
     <row r="253" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="8" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="B253" s="8" t="s">
         <v>78</v>
       </c>
       <c r="C253" s="8" t="s">
-        <v>1013</v>
+        <v>1016</v>
       </c>
       <c r="D253" s="8" t="s">
         <v>1017</v>
@@ -11228,16 +11237,16 @@
         <v>1019</v>
       </c>
       <c r="B254" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C254" s="8" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D254" s="8" t="s">
         <v>1020</v>
       </c>
-      <c r="D254" s="8" t="s">
+      <c r="E254" s="8" t="s">
         <v>1021</v>
-      </c>
-      <c r="E254" s="8" t="s">
-        <v>1022</v>
       </c>
       <c r="F254" s="12" t="s">
         <v>6</v>
@@ -11246,24 +11255,24 @@
         <v>98</v>
       </c>
       <c r="H254" s="8" t="s">
-        <v>1023</v>
+        <v>98</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="8" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="B255" s="8" t="s">
         <v>80</v>
       </c>
       <c r="C255" s="8" t="s">
+        <v>1023</v>
+      </c>
+      <c r="D255" s="8" t="s">
+        <v>1024</v>
+      </c>
+      <c r="E255" s="8" t="s">
         <v>1025</v>
-      </c>
-      <c r="D255" s="8" t="s">
-        <v>1026</v>
-      </c>
-      <c r="E255" s="8" t="s">
-        <v>1027</v>
       </c>
       <c r="F255" s="12" t="s">
         <v>6</v>
@@ -11272,24 +11281,24 @@
         <v>98</v>
       </c>
       <c r="H255" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="256" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="256" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="8" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B256" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C256" s="8" t="s">
         <v>1028</v>
       </c>
-      <c r="B256" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C256" s="8" t="s">
+      <c r="D256" s="8" t="s">
         <v>1029</v>
       </c>
-      <c r="D256" s="8" t="s">
+      <c r="E256" s="8" t="s">
         <v>1030</v>
-      </c>
-      <c r="E256" s="8" t="s">
-        <v>1031</v>
       </c>
       <c r="F256" s="12" t="s">
         <v>6</v>
@@ -11301,21 +11310,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="257" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="257" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="8" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B257" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C257" s="8" t="s">
         <v>1032</v>
       </c>
-      <c r="B257" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C257" s="8" t="s">
+      <c r="D257" s="8" t="s">
         <v>1033</v>
       </c>
-      <c r="D257" s="8" t="s">
+      <c r="E257" s="8" t="s">
         <v>1034</v>
-      </c>
-      <c r="E257" s="8" t="s">
-        <v>1035</v>
       </c>
       <c r="F257" s="12" t="s">
         <v>6</v>
@@ -11329,13 +11338,13 @@
     </row>
     <row r="258" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="8" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B258" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C258" s="8" t="s">
         <v>1036</v>
-      </c>
-      <c r="B258" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C258" s="8" t="s">
-        <v>18</v>
       </c>
       <c r="D258" s="8" t="s">
         <v>1037</v>
@@ -11353,10 +11362,36 @@
         <v>98</v>
       </c>
     </row>
+    <row r="259" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A259" s="8" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B259" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C259" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D259" s="8" t="s">
+        <v>1040</v>
+      </c>
+      <c r="E259" s="8" t="s">
+        <v>1041</v>
+      </c>
+      <c r="F259" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G259" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H259" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H258"/>
+  <autoFilter ref="A1:H259"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F458" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F459" type="list">
       <formula1>"Actual,Futuro,Asana ahora,Descartado"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat: transactional check-in RPC, inline check-in CTA, board settings+members, column reorder/rename, inline task composer, card assignee, Lista tab, mention pills, realtime comments
- Migration 20260911090000: save_checkin() SECURITY INVOKER RPC, profiles.preferences jsonb,
  comments + task_activity in realtime publication
- check-in: handleSave → single rpc call with try/catch; CTA card back inline (not sticky)
- boards: create/settings modal with access + members (board_members sync), archive;
  draggable column headers with per-user order (profiles.preferences), click-to-rename;
  inline Asana-style task composer; on-card assignee popover; objective chip removed; Lista tab
- comments: @mention pills while typing (highlight backdrop), serialize/deserialize helpers,
  useLiveRefetch realtime hook for task comments/activity and objective/KPI timelines
- docs: SCHEMA.md, inventory xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Inventario-funcionalidades-Kublau-OKR.xlsx
+++ b/docs/Inventario-funcionalidades-Kublau-OKR.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Inventario" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Inventario!$A$1:$H$259</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Inventario!$A$1:$H$267</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2163" uniqueCount="1042">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2227" uniqueCount="1069">
   <si>
     <t xml:space="preserve">Estado</t>
   </si>
@@ -2715,61 +2715,136 @@
     <t xml:space="preserve">F-218</t>
   </si>
   <si>
-    <t xml:space="preserve">CTA inline entre secciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mover el bloque calendario + CTA de vuelta al flujo, no fijo arriba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solicitud pendiente</t>
+    <t xml:space="preserve">Tab Lista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabla Tarea · Prioridad · Responsable · Fecha · Estado agrupada por sección (colapsable), con filtros/orden/agrupar y edición inline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-11</t>
   </si>
   <si>
     <t xml:space="preserve">F-219</t>
   </si>
   <si>
-    <t xml:space="preserve">Guardado atómico del check-in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un solo RPC transaccional en lugar de 6 escrituras</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hallazgo P0 de auditoría</t>
+    <t xml:space="preserve">Botón ⚙ Configuración del tablero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre, descripción, color, acceso (Público/Privado), miembros (agregar/quitar) y Archivar tablero</t>
   </si>
   <si>
     <t xml:space="preserve">F-220</t>
   </si>
   <si>
-    <t xml:space="preserve">Tabs Tablero / Lista / Calendario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Misma data en tres vistas; Lista con una columna por campo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lista y Calendario en fase posterior</t>
+    <t xml:space="preserve">Formulario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crear tablero con acceso y miembros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre, acceso público/privado, selección de miembros del workspace; avatares de miembros en el encabezado</t>
   </si>
   <si>
     <t xml:space="preserve">F-221</t>
   </si>
   <si>
-    <t xml:space="preserve">Botón "Opciones"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mostrar/ocultar campos en tarjeta, ocultar "Listo", subtareas</t>
+    <t xml:space="preserve">Reordenar columnas arrastrando el encabezado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orden guardado por usuario en profiles.preferences (cross-device)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-222</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editar nombre de columna al hacer clic en el título</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter guarda, Esc cancela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-223</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composer inline de tarea en la columna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarjeta con título enfocado + chips Prioridad / Asignado / Objetivo (opcionales); Enter guarda y permite seguir agregando</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-11 · formato Asana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-224</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarjeta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asignación directa desde la tarjeta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Círculo punteado con icono de usuario si no hay asignado; clic abre dropdown de miembros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-11 · chip de objetivo retirado de la tarjeta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-225</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciones como píldoras mientras se escribe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se muestra @Nombre resaltado; se serializa a @[Nombre](id) al guardar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-226</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comentarios y actividad en tiempo real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suscripción realtime a comments y task_activity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-227</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloque calendario + CTA inline entre hero y secciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ya no está fijo arriba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guardado atómico del check-in (RPC save_checkin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una transacción para checkin, objetivos, entradas, progress_logs y comentarios; try/catch con mensaje de error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementado 2026-09-11 · cierra P0 de auditoría</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-229</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reacciones 👍 y "Responder"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reacción rápida y respuesta en hilo</t>
   </si>
   <si>
     <t xml:space="preserve">Fase posterior</t>
   </si>
   <si>
-    <t xml:space="preserve">F-222</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reacciones 👍 y "Responder"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reacción rápida y respuesta en hilo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-223</t>
+    <t xml:space="preserve">F-230</t>
   </si>
   <si>
     <t xml:space="preserve">Tabs Tablero / Calendario en Mis Tareas</t>
@@ -2778,7 +2853,16 @@
     <t xml:space="preserve">Vistas alternativas del hub personal</t>
   </si>
   <si>
-    <t xml:space="preserve">F-224</t>
+    <t xml:space="preserve">F-231</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab Calendario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vista de calendario del tablero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-232</t>
   </si>
   <si>
     <t xml:space="preserve">Detalle de tarea</t>
@@ -2790,7 +2874,7 @@
     <t xml:space="preserve">Toggle de completado; tipos Tarea, Hito, Aprobación (Aprobar / Solicitar cambios / Rechazar) con "Convertir a"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-225</t>
+    <t xml:space="preserve">F-233</t>
   </si>
   <si>
     <t xml:space="preserve">Campo Estado personalizado</t>
@@ -2799,7 +2883,7 @@
     <t xml:space="preserve">On track / At risk / Off track / On hold como chips de color, separado de "completada"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-226</t>
+    <t xml:space="preserve">F-234</t>
   </si>
   <si>
     <t xml:space="preserve">Asignado (único) con typeahead</t>
@@ -2811,7 +2895,7 @@
     <t xml:space="preserve">Auto-agrega a "My tasks" del asignado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-227</t>
+    <t xml:space="preserve">F-235</t>
   </si>
   <si>
     <t xml:space="preserve">Colaboradores / seguidores</t>
@@ -2823,7 +2907,7 @@
     <t xml:space="preserve">Vista previa "N people will be notified"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-228</t>
+    <t xml:space="preserve">F-236</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha límite con fecha inicio, hora y recurrencia</t>
@@ -2832,7 +2916,7 @@
     <t xml:space="preserve">Selector de rango; vencida en rojo en la tarjeta</t>
   </si>
   <si>
-    <t xml:space="preserve">F-229</t>
+    <t xml:space="preserve">F-237</t>
   </si>
   <si>
     <t xml:space="preserve">Dependencias "Blocked by" / "Blocking"</t>
@@ -2841,7 +2925,7 @@
     <t xml:space="preserve">Vincula tareas entre proyectos; se dibujan en Timeline</t>
   </si>
   <si>
-    <t xml:space="preserve">F-230</t>
+    <t xml:space="preserve">F-238</t>
   </si>
   <si>
     <t xml:space="preserve">Multi-proyecto (multi-homing)</t>
@@ -2850,7 +2934,7 @@
     <t xml:space="preserve">Una tarea vive en N proyectos, cada uno con su selector de sección inline</t>
   </si>
   <si>
-    <t xml:space="preserve">F-231</t>
+    <t xml:space="preserve">F-239</t>
   </si>
   <si>
     <t xml:space="preserve">Campos personalizados por proyecto</t>
@@ -2862,7 +2946,7 @@
     <t xml:space="preserve">"Edit options" y "Auto-fill" (IA) desde el dropdown</t>
   </si>
   <si>
-    <t xml:space="preserve">F-232</t>
+    <t xml:space="preserve">F-240</t>
   </si>
   <si>
     <t xml:space="preserve">Descripción rich text</t>
@@ -2871,7 +2955,7 @@
     <t xml:space="preserve">Editor con formato</t>
   </si>
   <si>
-    <t xml:space="preserve">F-233</t>
+    <t xml:space="preserve">F-241</t>
   </si>
   <si>
     <t xml:space="preserve">Subtareas</t>
@@ -2880,7 +2964,7 @@
     <t xml:space="preserve">Lista inline con contador "0/1", asignado y fecha propios, detalle anidado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-234</t>
+    <t xml:space="preserve">F-242</t>
   </si>
   <si>
     <t xml:space="preserve">Adjuntos</t>
@@ -2889,7 +2973,7 @@
     <t xml:space="preserve">Archivos adjuntos a la tarea</t>
   </si>
   <si>
-    <t xml:space="preserve">F-235</t>
+    <t xml:space="preserve">F-243</t>
   </si>
   <si>
     <t xml:space="preserve">Likes, copiar enlace, pantalla completa, banner de privacidad</t>
@@ -2901,7 +2985,7 @@
     <t xml:space="preserve">"Make public"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-236</t>
+    <t xml:space="preserve">F-244</t>
   </si>
   <si>
     <t xml:space="preserve">Menú "…" de tarea</t>
@@ -2916,7 +3000,7 @@
     <t xml:space="preserve">IA: Summarize task, Draft subtasks</t>
   </si>
   <si>
-    <t xml:space="preserve">F-237</t>
+    <t xml:space="preserve">F-245</t>
   </si>
   <si>
     <t xml:space="preserve">Feed de actividad</t>
@@ -2931,10 +3015,7 @@
     <t xml:space="preserve">Eventos: creado, renombrado (show original), asignado, campo cambiado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-238</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Editor</t>
+    <t xml:space="preserve">F-246</t>
   </si>
   <si>
     <t xml:space="preserve">Rich text (títulos, listas, cita, código, tabla, imagen, embed, adjuntos)</t>
@@ -2943,7 +3024,7 @@
     <t xml:space="preserve">Comentarios con formato completo</t>
   </si>
   <si>
-    <t xml:space="preserve">F-239</t>
+    <t xml:space="preserve">F-247</t>
   </si>
   <si>
     <t xml:space="preserve">@mención de personas, tareas y proyectos</t>
@@ -2952,7 +3033,7 @@
     <t xml:space="preserve">Typeahead en todo el workspace</t>
   </si>
   <si>
-    <t xml:space="preserve">F-240</t>
+    <t xml:space="preserve">F-248</t>
   </si>
   <si>
     <t xml:space="preserve">Comentario</t>
@@ -2964,7 +3045,7 @@
     <t xml:space="preserve">Acciones sobre cada comentario</t>
   </si>
   <si>
-    <t xml:space="preserve">F-241</t>
+    <t xml:space="preserve">F-249</t>
   </si>
   <si>
     <t xml:space="preserve">IA: resumir tarea, recomendar ediciones</t>
@@ -2973,7 +3054,7 @@
     <t xml:space="preserve">Asistencia en el compositor</t>
   </si>
   <si>
-    <t xml:space="preserve">F-242</t>
+    <t xml:space="preserve">F-250</t>
   </si>
   <si>
     <t xml:space="preserve">Board</t>
@@ -2985,7 +3066,7 @@
     <t xml:space="preserve">"Add section" inline al final; menú: rename, add before/after, collapse, hide empty, add rule, delete</t>
   </si>
   <si>
-    <t xml:space="preserve">F-243</t>
+    <t xml:space="preserve">F-251</t>
   </si>
   <si>
     <t xml:space="preserve">Drag &amp; drop entre secciones y reorden de secciones</t>
@@ -2994,7 +3075,7 @@
     <t xml:space="preserve">Mover tarea = cambiar sección</t>
   </si>
   <si>
-    <t xml:space="preserve">F-244</t>
+    <t xml:space="preserve">F-252</t>
   </si>
   <si>
     <t xml:space="preserve">Menú contextual de tarjeta (click derecho)</t>
@@ -3003,7 +3084,7 @@
     <t xml:space="preserve">Duplicar, follow-up, completar, subtarea, convertir, abrir en pestaña, copiar enlace, eliminar, imagen de portada</t>
   </si>
   <si>
-    <t xml:space="preserve">F-245</t>
+    <t xml:space="preserve">F-253</t>
   </si>
   <si>
     <t xml:space="preserve">Tarjeta con campos configurables</t>
@@ -3012,7 +3093,7 @@
     <t xml:space="preserve">Chips (Priority), fecha, tag, avatar, contadores like/comentario/subtarea</t>
   </si>
   <si>
-    <t xml:space="preserve">F-246</t>
+    <t xml:space="preserve">F-254</t>
   </si>
   <si>
     <t xml:space="preserve">Vistas</t>
@@ -3027,7 +3108,7 @@
     <t xml:space="preserve">List: una columna por campo, "+" agrega campo</t>
   </si>
   <si>
-    <t xml:space="preserve">F-247</t>
+    <t xml:space="preserve">F-255</t>
   </si>
   <si>
     <t xml:space="preserve">Filtros rápidos + constructor apilable</t>
@@ -3036,7 +3117,7 @@
     <t xml:space="preserve">Incomplete, Completed, Just my tasks, Due this/next week; por asignado, fechas, tipo y cada campo personalizado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-248</t>
+    <t xml:space="preserve">F-256</t>
   </si>
   <si>
     <t xml:space="preserve">Ordenar por cualquier campo</t>
@@ -3045,7 +3126,7 @@
     <t xml:space="preserve">Fechas, asignado, likes, alfabético, cada campo personalizado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-249</t>
+    <t xml:space="preserve">F-257</t>
   </si>
   <si>
     <t xml:space="preserve">Agrupar por cualquier campo + subgrupo (swimlanes)</t>
@@ -3054,7 +3135,7 @@
     <t xml:space="preserve">Agrupación distinta de secciones con orden personalizado</t>
   </si>
   <si>
-    <t xml:space="preserve">F-250</t>
+    <t xml:space="preserve">F-258</t>
   </si>
   <si>
     <t xml:space="preserve">Panel "Options" por vista</t>
@@ -3063,7 +3144,7 @@
     <t xml:space="preserve">Mostrar/ocultar campos, subtareas colapsadas/expandidas, nombre/icono de vista</t>
   </si>
   <si>
-    <t xml:space="preserve">F-251</t>
+    <t xml:space="preserve">F-259</t>
   </si>
   <si>
     <t xml:space="preserve">Buscar en esta vista</t>
@@ -3072,7 +3153,7 @@
     <t xml:space="preserve">Búsqueda rápida</t>
   </si>
   <si>
-    <t xml:space="preserve">F-252</t>
+    <t xml:space="preserve">F-260</t>
   </si>
   <si>
     <t xml:space="preserve">Customize &gt; Fields</t>
@@ -3084,7 +3165,7 @@
     <t xml:space="preserve">Single-select, Multi-select, Date, People, Reference, Text, Number, Formula, ID, Timer, Time tracking, Rollup</t>
   </si>
   <si>
-    <t xml:space="preserve">F-253</t>
+    <t xml:space="preserve">F-261</t>
   </si>
   <si>
     <t xml:space="preserve">Biblioteca de campos del workspace</t>
@@ -3093,7 +3174,7 @@
     <t xml:space="preserve">Reusar campos entre proyectos; opciones con color; reordenar; IA "Recommend fields"</t>
   </si>
   <si>
-    <t xml:space="preserve">F-254</t>
+    <t xml:space="preserve">F-262</t>
   </si>
   <si>
     <t xml:space="preserve">Customize &gt; Rules</t>
@@ -3108,7 +3189,7 @@
     <t xml:space="preserve">Plantillas de reglas con IA</t>
   </si>
   <si>
-    <t xml:space="preserve">F-255</t>
+    <t xml:space="preserve">F-263</t>
   </si>
   <si>
     <t xml:space="preserve">Customize</t>
@@ -3120,7 +3201,7 @@
     <t xml:space="preserve">Intake y plantillas</t>
   </si>
   <si>
-    <t xml:space="preserve">F-256</t>
+    <t xml:space="preserve">F-264</t>
   </si>
   <si>
     <t xml:space="preserve">Menú de proyecto</t>
@@ -3132,7 +3213,7 @@
     <t xml:space="preserve">Gestión del proyecto</t>
   </si>
   <si>
-    <t xml:space="preserve">F-257</t>
+    <t xml:space="preserve">F-265</t>
   </si>
   <si>
     <t xml:space="preserve">My tasks / Inbox</t>
@@ -3144,7 +3225,7 @@
     <t xml:space="preserve">Lista personal con secciones automáticas ("Recently assigned")</t>
   </si>
   <si>
-    <t xml:space="preserve">F-258</t>
+    <t xml:space="preserve">F-266</t>
   </si>
   <si>
     <t xml:space="preserve">Widgets de conteo y gráficas</t>
@@ -3797,11 +3878,11 @@
       </c>
       <c r="C3" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A3,Inventario!$F:$F,"Actual")</f>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D3" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A3,Inventario!$F:$F,"Futuro")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A3,Inventario!$F:$F,"Asana ahora")</f>
@@ -4133,7 +4214,7 @@
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A17,Inventario!$F:$F,"Actual")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D17" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A17,Inventario!$F:$F,"Futuro")</f>
@@ -4145,7 +4226,7 @@
       </c>
       <c r="F17" s="8" t="n">
         <f aca="false">SUM(C17:E17)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4373,11 +4454,11 @@
       </c>
       <c r="C27" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A27,Inventario!$F:$F,"Actual")</f>
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D27" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A27,Inventario!$F:$F,"Futuro")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" s="8" t="n">
         <f aca="false">COUNTIFS(Inventario!$B:$B,$A27,Inventario!$F:$F,"Asana ahora")</f>
@@ -4385,7 +4466,7 @@
       </c>
       <c r="F27" s="8" t="n">
         <f aca="false">SUM(C27:E27)</f>
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4610,11 +4691,11 @@
       </c>
       <c r="C37" s="9" t="n">
         <f aca="false">SUM(C2:C36)</f>
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="D37" s="9" t="n">
         <f aca="false">SUM(D2:D36)</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E37" s="9" t="n">
         <f aca="false">SUM(E2:E36)</f>
@@ -4622,7 +4703,7 @@
       </c>
       <c r="F37" s="9" t="n">
         <f aca="false">SUM(F2:F36)</f>
-        <v>258</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -4641,7 +4722,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H259"/>
+  <dimension ref="A1:H267"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -10322,15 +10403,15 @@
         <v>894</v>
       </c>
     </row>
-    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="8" t="s">
         <v>895</v>
       </c>
       <c r="B219" s="8" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C219" s="8" t="s">
-        <v>136</v>
+        <v>805</v>
       </c>
       <c r="D219" s="8" t="s">
         <v>896</v>
@@ -10338,8 +10419,8 @@
       <c r="E219" s="8" t="s">
         <v>897</v>
       </c>
-      <c r="F219" s="11" t="s">
-        <v>4</v>
+      <c r="F219" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G219" s="8" t="s">
         <v>98</v>
@@ -10348,15 +10429,15 @@
         <v>898</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="8" t="s">
         <v>899</v>
       </c>
       <c r="B220" s="8" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C220" s="8" t="s">
-        <v>64</v>
+        <v>820</v>
       </c>
       <c r="D220" s="8" t="s">
         <v>900</v>
@@ -10364,25 +10445,25 @@
       <c r="E220" s="8" t="s">
         <v>901</v>
       </c>
-      <c r="F220" s="11" t="s">
-        <v>4</v>
+      <c r="F220" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G220" s="8" t="s">
-        <v>98</v>
+        <v>291</v>
       </c>
       <c r="H220" s="8" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="8" t="s">
         <v>902</v>
-      </c>
-    </row>
-    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A221" s="8" t="s">
-        <v>903</v>
       </c>
       <c r="B221" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C221" s="8" t="s">
-        <v>805</v>
+        <v>903</v>
       </c>
       <c r="D221" s="8" t="s">
         <v>904</v>
@@ -10390,181 +10471,181 @@
       <c r="E221" s="8" t="s">
         <v>905</v>
       </c>
-      <c r="F221" s="11" t="s">
-        <v>4</v>
+      <c r="F221" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G221" s="8" t="s">
-        <v>98</v>
+        <v>291</v>
       </c>
       <c r="H221" s="8" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="8" t="s">
         <v>906</v>
-      </c>
-    </row>
-    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A222" s="8" t="s">
-        <v>907</v>
       </c>
       <c r="B222" s="8" t="s">
         <v>68</v>
       </c>
       <c r="C222" s="8" t="s">
-        <v>820</v>
+        <v>805</v>
       </c>
       <c r="D222" s="8" t="s">
+        <v>907</v>
+      </c>
+      <c r="E222" s="8" t="s">
         <v>908</v>
       </c>
-      <c r="E222" s="8" t="s">
+      <c r="F222" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G222" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H222" s="8" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="8" t="s">
         <v>909</v>
       </c>
-      <c r="F222" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="G222" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="H222" s="8" t="s">
+      <c r="B223" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C223" s="8" t="s">
+        <v>805</v>
+      </c>
+      <c r="D223" s="8" t="s">
         <v>910</v>
       </c>
-    </row>
-    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A223" s="8" t="s">
+      <c r="E223" s="8" t="s">
         <v>911</v>
       </c>
-      <c r="B223" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C223" s="8" t="s">
-        <v>558</v>
-      </c>
-      <c r="D223" s="8" t="s">
+      <c r="F223" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G223" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="H223" s="8" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="8" t="s">
         <v>912</v>
       </c>
-      <c r="E223" s="8" t="s">
+      <c r="B224" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C224" s="8" t="s">
+        <v>805</v>
+      </c>
+      <c r="D224" s="8" t="s">
         <v>913</v>
       </c>
-      <c r="F223" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="G223" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="H223" s="8" t="s">
-        <v>910</v>
-      </c>
-    </row>
-    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A224" s="8" t="s">
+      <c r="E224" s="8" t="s">
         <v>914</v>
       </c>
-      <c r="B224" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C224" s="8" t="s">
-        <v>505</v>
-      </c>
-      <c r="D224" s="8" t="s">
+      <c r="F224" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G224" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="H224" s="8" t="s">
         <v>915</v>
-      </c>
-      <c r="E224" s="8" t="s">
-        <v>916</v>
-      </c>
-      <c r="F224" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="G224" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="H224" s="8" t="s">
-        <v>711</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="8" t="s">
+        <v>916</v>
+      </c>
+      <c r="B225" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C225" s="8" t="s">
         <v>917</v>
       </c>
-      <c r="B225" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C225" s="8" t="s">
+      <c r="D225" s="8" t="s">
         <v>918</v>
       </c>
-      <c r="D225" s="8" t="s">
+      <c r="E225" s="8" t="s">
         <v>919</v>
       </c>
-      <c r="E225" s="8" t="s">
+      <c r="F225" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G225" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="H225" s="8" t="s">
         <v>920</v>
       </c>
-      <c r="F225" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="G225" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="H225" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="226" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="8" t="s">
         <v>921</v>
       </c>
       <c r="B226" s="8" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="C226" s="8" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="D226" s="8" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="E226" s="8" t="s">
-        <v>923</v>
-      </c>
-      <c r="F226" s="12" t="s">
-        <v>6</v>
+        <v>924</v>
+      </c>
+      <c r="F226" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G226" s="8" t="s">
         <v>98</v>
       </c>
       <c r="H226" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="227" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="8" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B227" s="8" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="C227" s="8" t="s">
-        <v>918</v>
+        <v>666</v>
       </c>
       <c r="D227" s="8" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="E227" s="8" t="s">
-        <v>926</v>
-      </c>
-      <c r="F227" s="12" t="s">
-        <v>6</v>
+        <v>927</v>
+      </c>
+      <c r="F227" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G227" s="8" t="s">
         <v>98</v>
       </c>
       <c r="H227" s="8" t="s">
-        <v>927</v>
-      </c>
-    </row>
-    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="8" t="s">
         <v>928</v>
       </c>
       <c r="B228" s="8" t="s">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="C228" s="8" t="s">
-        <v>918</v>
+        <v>136</v>
       </c>
       <c r="D228" s="8" t="s">
         <v>929</v>
@@ -10572,40 +10653,40 @@
       <c r="E228" s="8" t="s">
         <v>930</v>
       </c>
-      <c r="F228" s="12" t="s">
-        <v>6</v>
+      <c r="F228" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="G228" s="8" t="s">
         <v>98</v>
       </c>
       <c r="H228" s="8" t="s">
-        <v>931</v>
+        <v>898</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="8" t="s">
+        <v>931</v>
+      </c>
+      <c r="B229" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C229" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D229" s="8" t="s">
         <v>932</v>
       </c>
-      <c r="B229" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C229" s="8" t="s">
-        <v>918</v>
-      </c>
-      <c r="D229" s="8" t="s">
+      <c r="E229" s="8" t="s">
         <v>933</v>
       </c>
-      <c r="E229" s="8" t="s">
+      <c r="F229" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G229" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H229" s="8" t="s">
         <v>934</v>
-      </c>
-      <c r="F229" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="G229" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="H229" s="8" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10613,10 +10694,10 @@
         <v>935</v>
       </c>
       <c r="B230" s="8" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="C230" s="8" t="s">
-        <v>918</v>
+        <v>558</v>
       </c>
       <c r="D230" s="8" t="s">
         <v>936</v>
@@ -10624,69 +10705,69 @@
       <c r="E230" s="8" t="s">
         <v>937</v>
       </c>
-      <c r="F230" s="12" t="s">
-        <v>6</v>
+      <c r="F230" s="11" t="s">
+        <v>4</v>
       </c>
       <c r="G230" s="8" t="s">
         <v>98</v>
       </c>
       <c r="H230" s="8" t="s">
-        <v>98</v>
+        <v>938</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="8" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="B231" s="8" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="C231" s="8" t="s">
-        <v>918</v>
+        <v>505</v>
       </c>
       <c r="D231" s="8" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="E231" s="8" t="s">
-        <v>940</v>
-      </c>
-      <c r="F231" s="12" t="s">
-        <v>6</v>
+        <v>941</v>
+      </c>
+      <c r="F231" s="11" t="s">
+        <v>4</v>
       </c>
       <c r="G231" s="8" t="s">
-        <v>98</v>
+        <v>4</v>
       </c>
       <c r="H231" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="232" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="8" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="B232" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C232" s="8" t="s">
-        <v>918</v>
+        <v>805</v>
       </c>
       <c r="D232" s="8" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="E232" s="8" t="s">
-        <v>943</v>
-      </c>
-      <c r="F232" s="12" t="s">
-        <v>6</v>
+        <v>944</v>
+      </c>
+      <c r="F232" s="11" t="s">
+        <v>4</v>
       </c>
       <c r="G232" s="8" t="s">
-        <v>98</v>
+        <v>4</v>
       </c>
       <c r="H232" s="8" t="s">
-        <v>944</v>
-      </c>
-    </row>
-    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="8" t="s">
         <v>945</v>
       </c>
@@ -10694,13 +10775,13 @@
         <v>70</v>
       </c>
       <c r="C233" s="8" t="s">
-        <v>918</v>
+        <v>946</v>
       </c>
       <c r="D233" s="8" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="E233" s="8" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="F233" s="12" t="s">
         <v>6</v>
@@ -10712,21 +10793,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="8" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="B234" s="8" t="s">
         <v>70</v>
       </c>
       <c r="C234" s="8" t="s">
-        <v>918</v>
+        <v>946</v>
       </c>
       <c r="D234" s="8" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="E234" s="8" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="F234" s="12" t="s">
         <v>6</v>
@@ -10738,21 +10819,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="8" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="B235" s="8" t="s">
         <v>70</v>
       </c>
       <c r="C235" s="8" t="s">
-        <v>918</v>
+        <v>946</v>
       </c>
       <c r="D235" s="8" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="E235" s="8" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="F235" s="12" t="s">
         <v>6</v>
@@ -10761,24 +10842,24 @@
         <v>98</v>
       </c>
       <c r="H235" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="236" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="8" t="s">
-        <v>954</v>
+        <v>956</v>
       </c>
       <c r="B236" s="8" t="s">
         <v>70</v>
       </c>
       <c r="C236" s="8" t="s">
-        <v>918</v>
+        <v>946</v>
       </c>
       <c r="D236" s="8" t="s">
-        <v>955</v>
+        <v>957</v>
       </c>
       <c r="E236" s="8" t="s">
-        <v>956</v>
+        <v>958</v>
       </c>
       <c r="F236" s="12" t="s">
         <v>6</v>
@@ -10787,24 +10868,24 @@
         <v>98</v>
       </c>
       <c r="H236" s="8" t="s">
-        <v>957</v>
-      </c>
-    </row>
-    <row r="237" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="8" t="s">
-        <v>958</v>
+        <v>960</v>
       </c>
       <c r="B237" s="8" t="s">
         <v>70</v>
       </c>
       <c r="C237" s="8" t="s">
-        <v>959</v>
+        <v>946</v>
       </c>
       <c r="D237" s="8" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="E237" s="8" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="F237" s="12" t="s">
         <v>6</v>
@@ -10813,24 +10894,24 @@
         <v>98</v>
       </c>
       <c r="H237" s="8" t="s">
-        <v>962</v>
-      </c>
-    </row>
-    <row r="238" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="8" t="s">
         <v>963</v>
       </c>
       <c r="B238" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C238" s="8" t="s">
+        <v>946</v>
+      </c>
+      <c r="D238" s="8" t="s">
         <v>964</v>
       </c>
-      <c r="D238" s="8" t="s">
+      <c r="E238" s="8" t="s">
         <v>965</v>
-      </c>
-      <c r="E238" s="8" t="s">
-        <v>966</v>
       </c>
       <c r="F238" s="12" t="s">
         <v>6</v>
@@ -10839,24 +10920,24 @@
         <v>98</v>
       </c>
       <c r="H238" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="8" t="s">
+        <v>966</v>
+      </c>
+      <c r="B239" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C239" s="8" t="s">
+        <v>946</v>
+      </c>
+      <c r="D239" s="8" t="s">
         <v>967</v>
       </c>
-    </row>
-    <row r="239" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A239" s="8" t="s">
+      <c r="E239" s="8" t="s">
         <v>968</v>
-      </c>
-      <c r="B239" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C239" s="8" t="s">
-        <v>969</v>
-      </c>
-      <c r="D239" s="8" t="s">
-        <v>970</v>
-      </c>
-      <c r="E239" s="8" t="s">
-        <v>971</v>
       </c>
       <c r="F239" s="12" t="s">
         <v>6</v>
@@ -10868,21 +10949,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="8" t="s">
-        <v>972</v>
+        <v>969</v>
       </c>
       <c r="B240" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C240" s="8" t="s">
-        <v>969</v>
+        <v>946</v>
       </c>
       <c r="D240" s="8" t="s">
-        <v>973</v>
+        <v>970</v>
       </c>
       <c r="E240" s="8" t="s">
-        <v>974</v>
+        <v>971</v>
       </c>
       <c r="F240" s="12" t="s">
         <v>6</v>
@@ -10891,24 +10972,24 @@
         <v>98</v>
       </c>
       <c r="H240" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="241" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="8" t="s">
+        <v>973</v>
+      </c>
+      <c r="B241" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C241" s="8" t="s">
+        <v>946</v>
+      </c>
+      <c r="D241" s="8" t="s">
+        <v>974</v>
+      </c>
+      <c r="E241" s="8" t="s">
         <v>975</v>
-      </c>
-      <c r="B241" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C241" s="8" t="s">
-        <v>976</v>
-      </c>
-      <c r="D241" s="8" t="s">
-        <v>977</v>
-      </c>
-      <c r="E241" s="8" t="s">
-        <v>978</v>
       </c>
       <c r="F241" s="12" t="s">
         <v>6</v>
@@ -10922,19 +11003,19 @@
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="8" t="s">
-        <v>979</v>
+        <v>976</v>
       </c>
       <c r="B242" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C242" s="8" t="s">
-        <v>969</v>
+        <v>946</v>
       </c>
       <c r="D242" s="8" t="s">
-        <v>980</v>
+        <v>977</v>
       </c>
       <c r="E242" s="8" t="s">
-        <v>981</v>
+        <v>978</v>
       </c>
       <c r="F242" s="12" t="s">
         <v>6</v>
@@ -10946,21 +11027,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="243" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="8" t="s">
-        <v>982</v>
+        <v>979</v>
       </c>
       <c r="B243" s="8" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C243" s="8" t="s">
-        <v>983</v>
+        <v>946</v>
       </c>
       <c r="D243" s="8" t="s">
-        <v>984</v>
+        <v>980</v>
       </c>
       <c r="E243" s="8" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
       <c r="F243" s="12" t="s">
         <v>6</v>
@@ -10974,19 +11055,19 @@
     </row>
     <row r="244" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="8" t="s">
-        <v>986</v>
+        <v>982</v>
       </c>
       <c r="B244" s="8" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C244" s="8" t="s">
+        <v>946</v>
+      </c>
+      <c r="D244" s="8" t="s">
         <v>983</v>
       </c>
-      <c r="D244" s="8" t="s">
-        <v>987</v>
-      </c>
       <c r="E244" s="8" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="F244" s="12" t="s">
         <v>6</v>
@@ -10995,24 +11076,24 @@
         <v>98</v>
       </c>
       <c r="H244" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="245" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="245" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="8" t="s">
+        <v>986</v>
+      </c>
+      <c r="B245" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C245" s="8" t="s">
+        <v>987</v>
+      </c>
+      <c r="D245" s="8" t="s">
+        <v>988</v>
+      </c>
+      <c r="E245" s="8" t="s">
         <v>989</v>
-      </c>
-      <c r="B245" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C245" s="8" t="s">
-        <v>983</v>
-      </c>
-      <c r="D245" s="8" t="s">
-        <v>990</v>
-      </c>
-      <c r="E245" s="8" t="s">
-        <v>991</v>
       </c>
       <c r="F245" s="12" t="s">
         <v>6</v>
@@ -11021,18 +11102,18 @@
         <v>98</v>
       </c>
       <c r="H245" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="246" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="8" t="s">
+        <v>991</v>
+      </c>
+      <c r="B246" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C246" s="8" t="s">
         <v>992</v>
-      </c>
-      <c r="B246" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C246" s="8" t="s">
-        <v>983</v>
       </c>
       <c r="D246" s="8" t="s">
         <v>993</v>
@@ -11047,18 +11128,18 @@
         <v>98</v>
       </c>
       <c r="H246" s="8" t="s">
-        <v>98</v>
+        <v>995</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="8" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="B247" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C247" s="8" t="s">
-        <v>996</v>
+        <v>922</v>
       </c>
       <c r="D247" s="8" t="s">
         <v>997</v>
@@ -11073,24 +11154,24 @@
         <v>98</v>
       </c>
       <c r="H247" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="8" t="s">
         <v>999</v>
       </c>
-    </row>
-    <row r="248" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A248" s="8" t="s">
+      <c r="B248" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C248" s="8" t="s">
+        <v>922</v>
+      </c>
+      <c r="D248" s="8" t="s">
         <v>1000</v>
       </c>
-      <c r="B248" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C248" s="8" t="s">
-        <v>820</v>
-      </c>
-      <c r="D248" s="8" t="s">
+      <c r="E248" s="8" t="s">
         <v>1001</v>
-      </c>
-      <c r="E248" s="8" t="s">
-        <v>1002</v>
       </c>
       <c r="F248" s="12" t="s">
         <v>6</v>
@@ -11102,15 +11183,15 @@
         <v>98</v>
       </c>
     </row>
-    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="249" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="8" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B249" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C249" s="8" t="s">
         <v>1003</v>
-      </c>
-      <c r="B249" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C249" s="8" t="s">
-        <v>820</v>
       </c>
       <c r="D249" s="8" t="s">
         <v>1004</v>
@@ -11128,15 +11209,15 @@
         <v>98</v>
       </c>
     </row>
-    <row r="250" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="8" t="s">
         <v>1006</v>
       </c>
       <c r="B250" s="8" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C250" s="8" t="s">
-        <v>820</v>
+        <v>922</v>
       </c>
       <c r="D250" s="8" t="s">
         <v>1007</v>
@@ -11159,16 +11240,16 @@
         <v>1009</v>
       </c>
       <c r="B251" s="8" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C251" s="8" t="s">
-        <v>820</v>
+        <v>1010</v>
       </c>
       <c r="D251" s="8" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="E251" s="8" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="F251" s="12" t="s">
         <v>6</v>
@@ -11180,21 +11261,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="252" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="8" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="B252" s="8" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C252" s="8" t="s">
-        <v>820</v>
+        <v>1010</v>
       </c>
       <c r="D252" s="8" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="E252" s="8" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="F252" s="12" t="s">
         <v>6</v>
@@ -11208,13 +11289,13 @@
     </row>
     <row r="253" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="8" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="B253" s="8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C253" s="8" t="s">
-        <v>1016</v>
+        <v>1010</v>
       </c>
       <c r="D253" s="8" t="s">
         <v>1017</v>
@@ -11232,15 +11313,15 @@
         <v>98</v>
       </c>
     </row>
-    <row r="254" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="8" t="s">
         <v>1019</v>
       </c>
       <c r="B254" s="8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C254" s="8" t="s">
-        <v>1016</v>
+        <v>1010</v>
       </c>
       <c r="D254" s="8" t="s">
         <v>1020</v>
@@ -11263,7 +11344,7 @@
         <v>1022</v>
       </c>
       <c r="B255" s="8" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C255" s="8" t="s">
         <v>1023</v>
@@ -11289,16 +11370,16 @@
         <v>1027</v>
       </c>
       <c r="B256" s="8" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C256" s="8" t="s">
+        <v>820</v>
+      </c>
+      <c r="D256" s="8" t="s">
         <v>1028</v>
       </c>
-      <c r="D256" s="8" t="s">
+      <c r="E256" s="8" t="s">
         <v>1029</v>
-      </c>
-      <c r="E256" s="8" t="s">
-        <v>1030</v>
       </c>
       <c r="F256" s="12" t="s">
         <v>6</v>
@@ -11310,21 +11391,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="257" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="8" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B257" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C257" s="8" t="s">
+        <v>820</v>
+      </c>
+      <c r="D257" s="8" t="s">
         <v>1031</v>
       </c>
-      <c r="B257" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C257" s="8" t="s">
+      <c r="E257" s="8" t="s">
         <v>1032</v>
-      </c>
-      <c r="D257" s="8" t="s">
-        <v>1033</v>
-      </c>
-      <c r="E257" s="8" t="s">
-        <v>1034</v>
       </c>
       <c r="F257" s="12" t="s">
         <v>6</v>
@@ -11338,19 +11419,19 @@
     </row>
     <row r="258" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B258" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C258" s="8" t="s">
+        <v>820</v>
+      </c>
+      <c r="D258" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="E258" s="8" t="s">
         <v>1035</v>
-      </c>
-      <c r="B258" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C258" s="8" t="s">
-        <v>1036</v>
-      </c>
-      <c r="D258" s="8" t="s">
-        <v>1037</v>
-      </c>
-      <c r="E258" s="8" t="s">
-        <v>1038</v>
       </c>
       <c r="F258" s="12" t="s">
         <v>6</v>
@@ -11364,19 +11445,19 @@
     </row>
     <row r="259" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="8" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
       <c r="B259" s="8" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C259" s="8" t="s">
-        <v>18</v>
+        <v>820</v>
       </c>
       <c r="D259" s="8" t="s">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="E259" s="8" t="s">
-        <v>1041</v>
+        <v>1038</v>
       </c>
       <c r="F259" s="12" t="s">
         <v>6</v>
@@ -11388,10 +11469,218 @@
         <v>98</v>
       </c>
     </row>
+    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="8" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B260" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C260" s="8" t="s">
+        <v>820</v>
+      </c>
+      <c r="D260" s="8" t="s">
+        <v>1040</v>
+      </c>
+      <c r="E260" s="8" t="s">
+        <v>1041</v>
+      </c>
+      <c r="F260" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G260" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H260" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="261" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="8" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B261" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C261" s="8" t="s">
+        <v>1043</v>
+      </c>
+      <c r="D261" s="8" t="s">
+        <v>1044</v>
+      </c>
+      <c r="E261" s="8" t="s">
+        <v>1045</v>
+      </c>
+      <c r="F261" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G261" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H261" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="262" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A262" s="8" t="s">
+        <v>1046</v>
+      </c>
+      <c r="B262" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C262" s="8" t="s">
+        <v>1043</v>
+      </c>
+      <c r="D262" s="8" t="s">
+        <v>1047</v>
+      </c>
+      <c r="E262" s="8" t="s">
+        <v>1048</v>
+      </c>
+      <c r="F262" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G262" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H262" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="263" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A263" s="8" t="s">
+        <v>1049</v>
+      </c>
+      <c r="B263" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C263" s="8" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D263" s="8" t="s">
+        <v>1051</v>
+      </c>
+      <c r="E263" s="8" t="s">
+        <v>1052</v>
+      </c>
+      <c r="F263" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G263" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H263" s="8" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="264" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A264" s="8" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B264" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C264" s="8" t="s">
+        <v>1055</v>
+      </c>
+      <c r="D264" s="8" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E264" s="8" t="s">
+        <v>1057</v>
+      </c>
+      <c r="F264" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G264" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H264" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="265" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A265" s="8" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B265" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C265" s="8" t="s">
+        <v>1059</v>
+      </c>
+      <c r="D265" s="8" t="s">
+        <v>1060</v>
+      </c>
+      <c r="E265" s="8" t="s">
+        <v>1061</v>
+      </c>
+      <c r="F265" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G265" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H265" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="266" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="8" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B266" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C266" s="8" t="s">
+        <v>1063</v>
+      </c>
+      <c r="D266" s="8" t="s">
+        <v>1064</v>
+      </c>
+      <c r="E266" s="8" t="s">
+        <v>1065</v>
+      </c>
+      <c r="F266" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G266" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H266" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="267" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A267" s="8" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B267" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C267" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D267" s="8" t="s">
+        <v>1067</v>
+      </c>
+      <c r="E267" s="8" t="s">
+        <v>1068</v>
+      </c>
+      <c r="F267" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G267" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H267" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H259"/>
+  <autoFilter ref="A1:H267"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F459" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F467" type="list">
       <formula1>"Actual,Futuro,Asana ahora,Descartado"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>